<commit_message>
D: stage-1 exclusion-sample adjudication done (177 rows: 114 advance / 63 exclude); confirmed-advance rates by code (TI04 27%, TI05 21%, others <=2.4%); PRE-007 re-screen scope pending A
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/04_screening/formal_2026-10-05_v0.9/ai_stage1/stage1_human_disagreements_for_D.xlsx
+++ b/04_screening/formal_2026-10-05_v0.9/ai_stage1/stage1_human_disagreements_for_D.xlsx
@@ -591,9 +591,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M2" s="4" t="inlineStr"/>
+      <c r="M2" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N2" s="4" t="inlineStr"/>
-      <c r="O2" s="4" t="inlineStr"/>
+      <c r="O2" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅列皮肤试验及哮喘特征，未明确非运动暴露；按 TI04 的指标/人群豁免推进。</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -648,9 +656,17 @@
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr"/>
-      <c r="M3" s="4" t="inlineStr"/>
+      <c r="M3" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N3" s="4" t="inlineStr"/>
-      <c r="O3" s="4" t="inlineStr"/>
+      <c r="O3" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cardiometabolic traits 与 determinants 未限定具体指标；不能证明全部结局非免疫，TI05 不成立。</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -709,9 +725,17 @@
           <t>TI05</t>
         </is>
       </c>
-      <c r="M4" s="4" t="inlineStr"/>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N4" s="4" t="inlineStr"/>
-      <c r="O4" s="4" t="inlineStr"/>
+      <c r="O4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名含运动及 fatigue recovery；恢复指标未限定，属 TI05 的 recovery 豁免。</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -770,9 +794,17 @@
           <t>TI05</t>
         </is>
       </c>
-      <c r="M5" s="4" t="inlineStr"/>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N5" s="4" t="inlineStr"/>
-      <c r="O5" s="4" t="inlineStr"/>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名涉及运动后肌痛，未限定为仅疼痛评分；按肌肉损伤/酸痛边界推进。</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -823,9 +855,17 @@
       </c>
       <c r="K6" s="3" t="inlineStr"/>
       <c r="L6" s="3" t="inlineStr"/>
-      <c r="M6" s="4" t="inlineStr"/>
+      <c r="M6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N6" s="4" t="inlineStr"/>
-      <c r="O6" s="4" t="inlineStr"/>
+      <c r="O6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">b-Cell 字形无法可靠区分 B 细胞与 β 细胞；不能确认仅非免疫结局，默认推进。</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -884,9 +924,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M7" s="4" t="inlineStr"/>
-      <c r="N7" s="4" t="inlineStr"/>
-      <c r="O7" s="4" t="inlineStr"/>
+      <c r="M7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">研究对象明确为灵芝真菌，属仅非人类生物研究；TI02 优先于热应激的 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -945,9 +997,17 @@
           <t>TI02</t>
         </is>
       </c>
-      <c r="M8" s="4" t="inlineStr"/>
+      <c r="M8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N8" s="4" t="inlineStr"/>
-      <c r="O8" s="4" t="inlineStr"/>
+      <c r="O8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bovine 修饰病毒名称，黏膜宿主未明；不能确认仅动物，且未明示非运动暴露，默认推进。</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -998,9 +1058,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M9" s="4" t="inlineStr"/>
-      <c r="N9" s="4" t="inlineStr"/>
-      <c r="O9" s="4" t="inlineStr"/>
+      <c r="M9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI04</t>
+        </is>
+      </c>
+      <c r="O9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">condom races 与 skills training 明确指安全性行为技能教育，非体育训练；按 TI04 排除。</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1059,9 +1131,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M10" s="4" t="inlineStr"/>
+      <c r="M10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N10" s="4" t="inlineStr"/>
-      <c r="O10" s="4" t="inlineStr"/>
+      <c r="O10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名为循环内皮细胞及心脏病人群，未明确非运动暴露；临床人群及缺少运动词不足以用 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1120,9 +1200,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M11" s="4" t="inlineStr"/>
+      <c r="M11" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N11" s="4" t="inlineStr"/>
-      <c r="O11" s="4" t="inlineStr"/>
+      <c r="O11" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅列哮喘免疫特征，report 未明确综述类型或非运动暴露；默认推进。</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1181,9 +1269,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M12" s="4" t="inlineStr"/>
+      <c r="M12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N12" s="4" t="inlineStr"/>
-      <c r="O12" s="4" t="inlineStr"/>
+      <c r="O12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名含抗氧化及氧化应激指标，risk factors 未具体限定；TI04/TI05 均不明确。</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1234,9 +1330,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M13" s="4" t="inlineStr"/>
-      <c r="N13" s="4" t="inlineStr"/>
-      <c r="O13" s="4" t="inlineStr"/>
+      <c r="M13" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N13" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI05</t>
+        </is>
+      </c>
+      <c r="O13" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">具名结局仅为骨骼肌镁异常，未列免疫或组学测量；juvenile 属病名，取 TI05。</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1295,9 +1403,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M14" s="4" t="inlineStr"/>
+      <c r="M14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N14" s="4" t="inlineStr"/>
-      <c r="O14" s="4" t="inlineStr"/>
+      <c r="O14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅比较细胞因子、消瘦状态及人群，未明确非运动研究暴露；按 TI04 豁免推进。</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1348,9 +1464,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M15" s="4" t="inlineStr"/>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N15" s="4" t="inlineStr"/>
-      <c r="O15" s="4" t="inlineStr"/>
+      <c r="O15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">training 未说明是技能教育还是体力训练；按训练情境豁免及不确定即推进原则保留。</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1409,9 +1533,21 @@
           <t>TI05</t>
         </is>
       </c>
-      <c r="M16" s="4" t="inlineStr"/>
-      <c r="N16" s="4" t="inlineStr"/>
-      <c r="O16" s="4" t="inlineStr"/>
+      <c r="M16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI05</t>
+        </is>
+      </c>
+      <c r="O16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">physical performance 可能涉及运动测试，TI04 不明确；具名结局仅血流动力学、血红蛋白及表现，取 TI05。</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1470,9 +1606,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M17" s="4" t="inlineStr"/>
+      <c r="M17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N17" s="4" t="inlineStr"/>
-      <c r="O17" s="4" t="inlineStr"/>
+      <c r="O17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅列 SLE 患者的心血管疾病，未说明研究暴露；临床人群不是题名排除理由。</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1531,9 +1675,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M18" s="4" t="inlineStr"/>
+      <c r="M18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N18" s="4" t="inlineStr"/>
-      <c r="O18" s="4" t="inlineStr"/>
+      <c r="O18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名在 with 处截断，且人体骨髓来源/参与者信息不完整；按截断题名默认推进规则保留。</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1592,9 +1744,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M19" s="4" t="inlineStr"/>
+      <c r="M19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N19" s="4" t="inlineStr"/>
-      <c r="O19" s="4" t="inlineStr"/>
+      <c r="O19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名含 IgE 及重组蛋白工具，未明确仅培养细胞或实际非运动暴露；默认推进。</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1653,9 +1813,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M20" s="4" t="inlineStr"/>
+      <c r="M20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N20" s="4" t="inlineStr"/>
-      <c r="O20" s="4" t="inlineStr"/>
+      <c r="O20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名含呼出 NO，未交代通气变化的诱发情境；不能确定无运动或炎症测量，推进。</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1714,9 +1882,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M21" s="4" t="inlineStr"/>
+      <c r="M21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N21" s="4" t="inlineStr"/>
-      <c r="O21" s="4" t="inlineStr"/>
+      <c r="O21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅为重症肌无力临床表型，未明确研究暴露；不因临床人群或疑似病例报告排除。</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1775,9 +1951,17 @@
           <t>TI05</t>
         </is>
       </c>
-      <c r="M22" s="4" t="inlineStr"/>
+      <c r="M22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N22" s="4" t="inlineStr"/>
-      <c r="O22" s="4" t="inlineStr"/>
+      <c r="O22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确骑行及肌痛，未限定为仅疼痛评分；按运动后酸痛边界推进。</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1836,9 +2020,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M23" s="4" t="inlineStr"/>
+      <c r="M23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N23" s="4" t="inlineStr"/>
-      <c r="O23" s="4" t="inlineStr"/>
+      <c r="O23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名为成人过敏人群的特异性 IgE 诊断指标，未明确非运动实验暴露；按 TI04 豁免推进。</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1893,9 +2085,17 @@
           <t>TI05</t>
         </is>
       </c>
-      <c r="M24" s="4" t="inlineStr"/>
+      <c r="M24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N24" s="4" t="inlineStr"/>
-      <c r="O24" s="4" t="inlineStr"/>
+      <c r="O24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">blood rheology 未限定为仅黏度或红细胞指标，存在可能相关血液内容；TI05 不明确。</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1954,9 +2154,17 @@
           <t>TI05</t>
         </is>
       </c>
-      <c r="M25" s="4" t="inlineStr"/>
+      <c r="M25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N25" s="4" t="inlineStr"/>
-      <c r="O25" s="4" t="inlineStr"/>
+      <c r="O25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名含 DOMS，未限定为仅症状评分；按运动后酸痛边界保留至摘要。</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2015,9 +2223,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M26" s="4" t="inlineStr"/>
+      <c r="M26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N26" s="4" t="inlineStr"/>
-      <c r="O26" s="4" t="inlineStr"/>
+      <c r="O26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅描述沙门菌与中性粒细胞的免疫过程，未明示宿主或实验暴露；TI02/TI04 不明确。</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2076,9 +2292,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M27" s="4" t="inlineStr"/>
+      <c r="M27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N27" s="4" t="inlineStr"/>
-      <c r="O27" s="4" t="inlineStr"/>
+      <c r="O27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名含 IgE 反应及蛋白结构，未明确人体来源或实际非运动暴露；默认推进。</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2137,9 +2361,17 @@
           <t>TI05</t>
         </is>
       </c>
-      <c r="M28" s="4" t="inlineStr"/>
+      <c r="M28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N28" s="4" t="inlineStr"/>
-      <c r="O28" s="4" t="inlineStr"/>
+      <c r="O28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名含 exercise capacity 及未限定的 response rate，且末尾截断；不能确认 TI05，推进。</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2198,9 +2430,21 @@
           <t>TI05</t>
         </is>
       </c>
-      <c r="M29" s="4" t="inlineStr"/>
-      <c r="N29" s="4" t="inlineStr"/>
-      <c r="O29" s="4" t="inlineStr"/>
+      <c r="M29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI05</t>
+        </is>
+      </c>
+      <c r="O29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">anaerobic threshold 本身涉及运动测试，减重方式未明，TI04 不成立；具名结局仅无氧阈，取 TI05。</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2259,9 +2503,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M30" s="4" t="inlineStr"/>
+      <c r="M30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N30" s="4" t="inlineStr"/>
-      <c r="O30" s="4" t="inlineStr"/>
+      <c r="O30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅列特异性 IgE 与过敏表型，未明确研究暴露；按 TI04 的指标/人群豁免推进。</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2312,9 +2564,21 @@
           <t>TI05</t>
         </is>
       </c>
-      <c r="M31" s="4" t="inlineStr"/>
-      <c r="N31" s="4" t="inlineStr"/>
-      <c r="O31" s="4" t="inlineStr"/>
+      <c r="M31" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N31" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI05</t>
+        </is>
+      </c>
+      <c r="O31" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确运动情境，但具名结局仅支气管收缩，未列免疫/炎症测量；按气道症状边界取 TI05。</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2373,9 +2637,17 @@
           <t>TI05</t>
         </is>
       </c>
-      <c r="M32" s="4" t="inlineStr"/>
+      <c r="M32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N32" s="4" t="inlineStr"/>
-      <c r="O32" s="4" t="inlineStr"/>
+      <c r="O32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名含运动及具名蛋白 FGF21，非仅列激素浓度；按 TI05 的可能相关蛋白豁免推进。</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2434,9 +2706,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M33" s="4" t="inlineStr"/>
+      <c r="M33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N33" s="4" t="inlineStr"/>
-      <c r="O33" s="4" t="inlineStr"/>
+      <c r="O33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">综合诊断 work-up 未限定检测项目或暴露；疾病人群及缺少运动词不能构成 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2495,9 +2775,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M34" s="4" t="inlineStr"/>
-      <c r="N34" s="4" t="inlineStr"/>
-      <c r="O34" s="4" t="inlineStr"/>
+      <c r="M34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确仅李斯特菌菌株的生长、侵入及菌株竞争；competition 非体育情境，取 TI02。</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2556,9 +2848,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M35" s="4" t="inlineStr"/>
+      <c r="M35" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N35" s="4" t="inlineStr"/>
-      <c r="O35" s="4" t="inlineStr"/>
+      <c r="O35" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名泛指重症疾病中的分子机制，未明确实际暴露及测量；临床背景不能直接作 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2617,9 +2917,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M36" s="4" t="inlineStr"/>
+      <c r="M36" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N36" s="4" t="inlineStr"/>
-      <c r="O36" s="4" t="inlineStr"/>
+      <c r="O36" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名含免疫蛋白 MIF，未说明心肌缺血是否由运动诱发；不能确认 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2678,9 +2986,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M37" s="4" t="inlineStr"/>
+      <c r="M37" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N37" s="4" t="inlineStr"/>
-      <c r="O37" s="4" t="inlineStr"/>
+      <c r="O37" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">controlled ischemia 未说明诱发方式，rheologic variables 未具体限定；TI04/TI05 不明确。</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2739,9 +3055,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M38" s="4" t="inlineStr"/>
+      <c r="M38" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N38" s="4" t="inlineStr"/>
-      <c r="O38" s="4" t="inlineStr"/>
+      <c r="O38" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名含白细胞流变学，受控冠脉缺血的诱发方式未明；不能确认 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2800,9 +3124,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M39" s="4" t="inlineStr"/>
+      <c r="M39" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N39" s="4" t="inlineStr"/>
-      <c r="O39" s="4" t="inlineStr"/>
+      <c r="O39" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名含 Hippo/YAP1 通路及免疫疾病，未明示实验暴露或仅培养细胞；默认推进。</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2861,9 +3193,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M40" s="4" t="inlineStr"/>
+      <c r="M40" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N40" s="4" t="inlineStr"/>
-      <c r="O40" s="4" t="inlineStr"/>
+      <c r="O40" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名为过敏原蛋白及交叉反应，植物名指蛋白来源；未明确仅非人类对象或非运动暴露。</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2922,9 +3262,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M41" s="4" t="inlineStr"/>
+      <c r="M41" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N41" s="4" t="inlineStr"/>
-      <c r="O41" s="4" t="inlineStr"/>
+      <c r="O41" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名描述 irisin 的分子功能，未明示给药、物种或培养实验；不能推定 TI02/TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2983,9 +3331,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M42" s="4" t="inlineStr"/>
-      <c r="N42" s="4" t="inlineStr"/>
-      <c r="O42" s="4" t="inlineStr"/>
+      <c r="M42" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N42" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O42" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确鉴定由鞘氨醇单胞菌产生的虾青素及衍生物，研究对象仅细菌产物；取 TI02。</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3044,9 +3404,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M43" s="4" t="inlineStr"/>
+      <c r="M43" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N43" s="4" t="inlineStr"/>
-      <c r="O43" s="4" t="inlineStr"/>
+      <c r="O43" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名含人群及未限定的 allostatic load，族群/贫困比较不等于明确非运动暴露；默认推进。</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3105,9 +3473,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M44" s="4" t="inlineStr"/>
+      <c r="M44" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N44" s="4" t="inlineStr"/>
-      <c r="O44" s="4" t="inlineStr"/>
+      <c r="O44" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅列食物过敏患者、过敏原及临床特征；未明确非运动研究暴露，TI04 不成立。</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3166,9 +3542,17 @@
           <t>TI05</t>
         </is>
       </c>
-      <c r="M45" s="4" t="inlineStr"/>
+      <c r="M45" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N45" s="4" t="inlineStr"/>
-      <c r="O45" s="4" t="inlineStr"/>
+      <c r="O45" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名未限定 physical/functional impairments 的检测，且含 infection；不足以确认全部结局非免疫。</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3227,9 +3611,21 @@
           <t>TI02</t>
         </is>
       </c>
-      <c r="M46" s="4" t="inlineStr"/>
-      <c r="N46" s="4" t="inlineStr"/>
-      <c r="O46" s="4" t="inlineStr"/>
+      <c r="M46" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N46" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI04</t>
+        </is>
+      </c>
+      <c r="O46" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mice 与 humans 同现，按 TI02 豁免保留该维度；暴露明确为烧伤且无运动情境，取 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3288,9 +3684,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M47" s="4" t="inlineStr"/>
+      <c r="M47" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N47" s="4" t="inlineStr"/>
-      <c r="O47" s="4" t="inlineStr"/>
+      <c r="O47" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅比较过敏表型的地域差异，未明确实验暴露；缺少运动词不足以用 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3349,9 +3753,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M48" s="4" t="inlineStr"/>
+      <c r="M48" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N48" s="4" t="inlineStr"/>
-      <c r="O48" s="4" t="inlineStr"/>
+      <c r="O48" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名含尿酸及未限定的 clinical outcomes，未明确研究暴露；不能由临床人群直接排除。</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3406,9 +3818,21 @@
           <t>TI05</t>
         </is>
       </c>
-      <c r="M49" s="4" t="inlineStr"/>
-      <c r="N49" s="4" t="inlineStr"/>
-      <c r="O49" s="4" t="inlineStr"/>
+      <c r="M49" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N49" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI05</t>
+        </is>
+      </c>
+      <c r="O49" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">具名测量为红外成像的皮肤温度变化，DOMS 是比较情境；未列免疫/组学结局，取 TI05。</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3467,9 +3891,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M50" s="4" t="inlineStr"/>
-      <c r="N50" s="4" t="inlineStr"/>
-      <c r="O50" s="4" t="inlineStr"/>
+      <c r="M50" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N50" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI04</t>
+        </is>
+      </c>
+      <c r="O50" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">training camp 是应对压力的比喻，题名明确心理韧性/疫情应激调查；无体力活动情境，取 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3528,9 +3964,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M51" s="4" t="inlineStr"/>
+      <c r="M51" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N51" s="4" t="inlineStr"/>
-      <c r="O51" s="4" t="inlineStr"/>
+      <c r="O51" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅比较成人食物过敏反应，未明确实际暴露及运动共因子；按 TI04 豁免推进。</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3589,9 +4033,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M52" s="4" t="inlineStr"/>
+      <c r="M52" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N52" s="4" t="inlineStr"/>
-      <c r="O52" s="4" t="inlineStr"/>
+      <c r="O52" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅列过敏原致敏分组及临床特征，未明确研究暴露；不以缺少运动词排除。</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3650,9 +4102,17 @@
           <t>TI01</t>
         </is>
       </c>
-      <c r="M53" s="4" t="inlineStr"/>
+      <c r="M53" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N53" s="4" t="inlineStr"/>
-      <c r="O53" s="4" t="inlineStr"/>
+      <c r="O53" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名只有疾病名称，未说明研究暴露、测量结局或来源类型；默认推进。</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3711,9 +4171,21 @@
           <t>TI05</t>
         </is>
       </c>
-      <c r="M54" s="4" t="inlineStr"/>
-      <c r="N54" s="4" t="inlineStr"/>
-      <c r="O54" s="4" t="inlineStr"/>
+      <c r="M54" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N54" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI05</t>
+        </is>
+      </c>
+      <c r="O54" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Long COVID 属临床人群描述，不能用 TI04；具名测量仅自主神经功能及 HRV，取 TI05。</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3772,9 +4244,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M55" s="4" t="inlineStr"/>
+      <c r="M55" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N55" s="4" t="inlineStr"/>
-      <c r="O55" s="4" t="inlineStr"/>
+      <c r="O55" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">蔗糖工人的 work-recovery 可含体力劳动，且题名含 inflammation；不能确认 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -3833,9 +4313,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M56" s="4" t="inlineStr"/>
+      <c r="M56" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N56" s="4" t="inlineStr"/>
-      <c r="O56" s="4" t="inlineStr"/>
+      <c r="O56" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名为人体脑转录组及神经免疫通路比较，race 指族群；未明确非运动实验暴露，推进。</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -3894,9 +4382,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M57" s="4" t="inlineStr"/>
+      <c r="M57" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N57" s="4" t="inlineStr"/>
-      <c r="O57" s="4" t="inlineStr"/>
+      <c r="O57" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名描述 MIF-ACKR3 分子机制，未明示给药或仅细胞培养；临床背景不足以用 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -3955,9 +4451,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M58" s="4" t="inlineStr"/>
+      <c r="M58" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N58" s="4" t="inlineStr"/>
-      <c r="O58" s="4" t="inlineStr"/>
+      <c r="O58" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">环境丰富化及 stress 未明确限定为非体力活动/心理应激，且含微生物组；默认推进。</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -4016,9 +4520,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M59" s="4" t="inlineStr"/>
+      <c r="M59" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N59" s="4" t="inlineStr"/>
-      <c r="O59" s="4" t="inlineStr"/>
+      <c r="O59" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名含免疫球蛋白及酶活性，只列康复人群而未指明暴露；按 TI04 豁免推进。</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -4073,9 +4585,17 @@
         </is>
       </c>
       <c r="L60" s="3" t="inlineStr"/>
-      <c r="M60" s="4" t="inlineStr"/>
+      <c r="M60" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N60" s="4" t="inlineStr"/>
-      <c r="O60" s="4" t="inlineStr"/>
+      <c r="O60" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅比较职业人群及未限定的心血管风险，未明确非运动暴露或全非免疫指标；推进。</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -4134,9 +4654,17 @@
           <t>TI05</t>
         </is>
       </c>
-      <c r="M61" s="4" t="inlineStr"/>
+      <c r="M61" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N61" s="4" t="inlineStr"/>
-      <c r="O61" s="4" t="inlineStr"/>
+      <c r="O61" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名含 DOMS，运动后酸痛提供可能运动情境且未限定为评分；TI04/TI05 不明确。</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -4187,9 +4715,17 @@
           <t>TI05</t>
         </is>
       </c>
-      <c r="M62" s="4" t="inlineStr"/>
+      <c r="M62" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N62" s="4" t="inlineStr"/>
-      <c r="O62" s="4" t="inlineStr"/>
+      <c r="O62" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确运动与 biomarkers，未限定检测为仅矿物浓度；按 TI05 的生物标志物豁免推进。</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -4248,9 +4784,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M63" s="4" t="inlineStr"/>
-      <c r="N63" s="4" t="inlineStr"/>
-      <c r="O63" s="4" t="inlineStr"/>
+      <c r="M63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI04</t>
+        </is>
+      </c>
+      <c r="O63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">病例报告本身属 TI01 豁免；暴露明确为 IVIg/化疗且无运动情境，按 TI04 排除。</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -4309,9 +4857,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M64" s="4" t="inlineStr"/>
+      <c r="M64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N64" s="4" t="inlineStr"/>
-      <c r="O64" s="4" t="inlineStr"/>
+      <c r="O64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名为支气管肺泡灌洗特征及免疫疾病比较，未明确非运动研究暴露；默认推进。</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -4362,9 +4918,17 @@
           <t>TI05</t>
         </is>
       </c>
-      <c r="M65" s="4" t="inlineStr"/>
+      <c r="M65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N65" s="4" t="inlineStr"/>
-      <c r="O65" s="4" t="inlineStr"/>
+      <c r="O65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">immunity to coronary heart disease 的防病/免疫含义及具体指标未明；不能确认全非免疫结局。</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -4423,9 +4987,17 @@
           <t>TI05</t>
         </is>
       </c>
-      <c r="M66" s="4" t="inlineStr"/>
+      <c r="M66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N66" s="4" t="inlineStr"/>
-      <c r="O66" s="4" t="inlineStr"/>
+      <c r="O66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确运动及受体/cAMP 分子系统，非仅激素浓度；按可能相关蛋白内容的 TI05 豁免推进。</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -4484,9 +5056,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M67" s="4" t="inlineStr"/>
-      <c r="N67" s="4" t="inlineStr"/>
-      <c r="O67" s="4" t="inlineStr"/>
+      <c r="M67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI04</t>
+        </is>
+      </c>
+      <c r="O67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">人体造血祖细胞可来自人样本，TI02 不明确；题名明确药物毒性暴露且无运动，取 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -4545,9 +5129,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M68" s="4" t="inlineStr"/>
-      <c r="N68" s="4" t="inlineStr"/>
-      <c r="O68" s="4" t="inlineStr"/>
+      <c r="M68" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N68" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI04</t>
+        </is>
+      </c>
+      <c r="O68" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">summary 未明确属于封闭清单中的综述类型；题名明确药物试验且无运动情境，取 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -4606,9 +5202,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M69" s="4" t="inlineStr"/>
+      <c r="M69" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N69" s="4" t="inlineStr"/>
-      <c r="O69" s="4" t="inlineStr"/>
+      <c r="O69" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名含基因变异及血液病表型，未明示研究暴露；临床人群与疑似病例报告不单独排除。</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -4667,9 +5271,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M70" s="4" t="inlineStr"/>
+      <c r="M70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N70" s="4" t="inlineStr"/>
-      <c r="O70" s="4" t="inlineStr"/>
+      <c r="O70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅称转化模型，未明确物种、培养细胞或研究暴露；不能推定 TI02/TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -4728,9 +5340,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M71" s="4" t="inlineStr"/>
+      <c r="M71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N71" s="4" t="inlineStr"/>
-      <c r="O71" s="4" t="inlineStr"/>
+      <c r="O71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名含机械感知及免疫稳态，未明确实际刺激方式或物种；不能确认非运动暴露。</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -4789,9 +5409,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M72" s="4" t="inlineStr"/>
+      <c r="M72" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N72" s="4" t="inlineStr"/>
-      <c r="O72" s="4" t="inlineStr"/>
+      <c r="O72" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名为临床诊断表型，未明确研究暴露或非免疫测量；病例性质不单独构成 TI01。</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -4850,9 +5478,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M73" s="4" t="inlineStr"/>
-      <c r="N73" s="4" t="inlineStr"/>
-      <c r="O73" s="4" t="inlineStr"/>
+      <c r="M73" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N73" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI04</t>
+        </is>
+      </c>
+      <c r="O73" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">病例报告属 TI01 豁免；题名明确针刀/中医治疗且无运动情境，按 TI04 排除。</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -4911,9 +5551,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M74" s="4" t="inlineStr"/>
+      <c r="M74" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N74" s="4" t="inlineStr"/>
-      <c r="O74" s="4" t="inlineStr"/>
+      <c r="O74" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名描述 IL-6 的酶调节功能，未明示外源给药或实际实验暴露；不能推定 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -4972,9 +5620,21 @@
           <t>TI02</t>
         </is>
       </c>
-      <c r="M75" s="4" t="inlineStr"/>
-      <c r="N75" s="4" t="inlineStr"/>
-      <c r="O75" s="4" t="inlineStr"/>
+      <c r="M75" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N75" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O75" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确香蕉在镰刀菌感染中的转录组，研究对象仅植物/真菌；取 TI02。</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -5033,9 +5693,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M76" s="4" t="inlineStr"/>
+      <c r="M76" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N76" s="4" t="inlineStr"/>
-      <c r="O76" s="4" t="inlineStr"/>
+      <c r="O76" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名含巨噬细胞、抗炎及具名信号通路，未明示给药/物种/培养细胞；默认推进。</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -5094,9 +5762,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M77" s="4" t="inlineStr"/>
+      <c r="M77" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N77" s="4" t="inlineStr"/>
-      <c r="O77" s="4" t="inlineStr"/>
+      <c r="O77" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名为免疫疾病的诊断表型，未明确研究暴露；临床人群或疑似病例不能单独排除。</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -5155,9 +5831,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M78" s="4" t="inlineStr"/>
+      <c r="M78" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N78" s="4" t="inlineStr"/>
-      <c r="O78" s="4" t="inlineStr"/>
+      <c r="O78" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIS-C 是疾病缩写，题名未明示仅未成年队列或具体随访测量；TI03/TI05 不明确。</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -5216,9 +5900,21 @@
           <t>TI03</t>
         </is>
       </c>
-      <c r="M79" s="4" t="inlineStr"/>
-      <c r="N79" s="4" t="inlineStr"/>
-      <c r="O79" s="4" t="inlineStr"/>
+      <c r="M79" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N79" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI03</t>
+        </is>
+      </c>
+      <c r="O79" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">病例报告属 TI01 豁免；题名明确仅 adolescents，按 TI03 排除并优先于 TI05。</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -5277,9 +5973,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M80" s="4" t="inlineStr"/>
+      <c r="M80" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N80" s="4" t="inlineStr"/>
-      <c r="O80" s="4" t="inlineStr"/>
+      <c r="O80" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">race 指族群，题名仅比较疾病表现与人群特征；未明确非运动研究暴露，推进。</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -5338,9 +6042,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M81" s="4" t="inlineStr"/>
-      <c r="N81" s="4" t="inlineStr"/>
-      <c r="O81" s="4" t="inlineStr"/>
+      <c r="M81" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N81" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O81" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确鉴定缺失麦醇溶蛋白的植物 wheat lines，非人体研究；取 TI02。</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -5399,9 +6115,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M82" s="4" t="inlineStr"/>
+      <c r="M82" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N82" s="4" t="inlineStr"/>
-      <c r="O82" s="4" t="inlineStr"/>
+      <c r="O82" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名为患者的蛋白过敏综合征，case report 属 TI01 豁免；无其他明确封闭理由，推进。</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -5452,9 +6176,21 @@
           <t>TI05</t>
         </is>
       </c>
-      <c r="M83" s="4" t="inlineStr"/>
-      <c r="N83" s="4" t="inlineStr"/>
-      <c r="O83" s="4" t="inlineStr"/>
+      <c r="M83" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N83" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI05</t>
+        </is>
+      </c>
+      <c r="O83" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">可读的英文题名将结局明确限定为 pain intensity 及 range of motion；按疼痛评分/功能边界取 TI05。</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -5513,9 +6249,21 @@
           <t>TI02</t>
         </is>
       </c>
-      <c r="M84" s="4" t="inlineStr"/>
-      <c r="N84" s="4" t="inlineStr"/>
-      <c r="O84" s="4" t="inlineStr"/>
+      <c r="M84" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N84" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O84" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确 animal model，研究对象仅动物；TI02 优先于药物/骨结局的 TI04/TI05。</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -5574,9 +6322,17 @@
           <t>TI05</t>
         </is>
       </c>
-      <c r="M85" s="4" t="inlineStr"/>
+      <c r="M85" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N85" s="4" t="inlineStr"/>
-      <c r="O85" s="4" t="inlineStr"/>
+      <c r="O85" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确抗阻运动、运动员及 DOMS，未限定为仅症状评分；按酸痛边界推进。</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -5635,9 +6391,17 @@
           <t>TI05</t>
         </is>
       </c>
-      <c r="M86" s="4" t="inlineStr"/>
+      <c r="M86" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N86" s="4" t="inlineStr"/>
-      <c r="O86" s="4" t="inlineStr"/>
+      <c r="O86" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确训练及具名蛋白 BDNF；按 TI05 的可能相关蛋白豁免推进，临床人群不单独排除。</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -5696,9 +6460,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M87" s="4" t="inlineStr"/>
+      <c r="M87" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N87" s="4" t="inlineStr"/>
-      <c r="O87" s="4" t="inlineStr"/>
+      <c r="O87" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅列临床感染个案，未明确研究暴露；病例报告属 TI01 豁免，默认推进。</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -5757,9 +6529,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M88" s="4" t="inlineStr"/>
+      <c r="M88" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N88" s="4" t="inlineStr"/>
-      <c r="O88" s="4" t="inlineStr"/>
+      <c r="O88" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名未列具体病因暴露、检测指标或来源类型；不能由疾病主题推定 TI01/TI04/TI05。</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -5818,9 +6598,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M89" s="4" t="inlineStr"/>
-      <c r="N89" s="4" t="inlineStr"/>
-      <c r="O89" s="4" t="inlineStr"/>
+      <c r="M89" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N89" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O89" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确水稻对黄单胞菌的转录反应，race 指菌株；研究对象仅非人类生物，取 TI02。</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -5879,9 +6671,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M90" s="4" t="inlineStr"/>
-      <c r="N90" s="4" t="inlineStr"/>
-      <c r="O90" s="4" t="inlineStr"/>
+      <c r="M90" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N90" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI05</t>
+        </is>
+      </c>
+      <c r="O90" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">病例报告属 TI01 豁免，疾病人群不能作 TI04；具名结局仅肌电活动变化，取 TI05。</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -5940,9 +6744,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M91" s="4" t="inlineStr"/>
-      <c r="N91" s="4" t="inlineStr"/>
-      <c r="O91" s="4" t="inlineStr"/>
+      <c r="M91" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N91" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI05</t>
+        </is>
+      </c>
+      <c r="O91" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">妊娠及疾病名称是人群描述，TI04 不明确；具名结局仅背痛及功能状态，取 TI05。</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -6001,9 +6817,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M92" s="4" t="inlineStr"/>
+      <c r="M92" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N92" s="4" t="inlineStr"/>
-      <c r="O92" s="4" t="inlineStr"/>
+      <c r="O92" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅为食物过敏的组分诊断，未明示实际非运动暴露；按 TI04 豁免推进。</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -6062,9 +6886,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M93" s="4" t="inlineStr"/>
-      <c r="N93" s="4" t="inlineStr"/>
-      <c r="O93" s="4" t="inlineStr"/>
+      <c r="M93" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N93" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O93" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确商业小麦中的蛋白组及表位分析，研究对象仅植物蛋白；取 TI02。</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -6115,9 +6951,17 @@
           <t>TI05</t>
         </is>
       </c>
-      <c r="M94" s="4" t="inlineStr"/>
+      <c r="M94" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N94" s="4" t="inlineStr"/>
-      <c r="O94" s="4" t="inlineStr"/>
+      <c r="O94" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确瑜伽运动及肌肉撕裂，属可能相关肌肉损伤；病例报告为 TI01 豁免，推进。</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -6176,9 +7020,17 @@
           <t>TI05</t>
         </is>
       </c>
-      <c r="M95" s="4" t="inlineStr"/>
+      <c r="M95" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N95" s="4" t="inlineStr"/>
-      <c r="O95" s="4" t="inlineStr"/>
+      <c r="O95" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确运动，brain microvascular alterations 未限定具体测量；不能确认所有结局非免疫。</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -6237,9 +7089,17 @@
           <t>TI05</t>
         </is>
       </c>
-      <c r="M96" s="4" t="inlineStr"/>
+      <c r="M96" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N96" s="4" t="inlineStr"/>
-      <c r="O96" s="4" t="inlineStr"/>
+      <c r="O96" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名有骨骼肌收缩，anabolic response 未限定具体指标；临床感染背景不作 TI04，推进。</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -6298,9 +7158,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M97" s="4" t="inlineStr"/>
+      <c r="M97" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N97" s="4" t="inlineStr"/>
-      <c r="O97" s="4" t="inlineStr"/>
+      <c r="O97" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅列临床及病理发现，未明确实际暴露或具体非免疫测量；默认推进。</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -6359,9 +7227,21 @@
           <t>TI05</t>
         </is>
       </c>
-      <c r="M98" s="4" t="inlineStr"/>
-      <c r="N98" s="4" t="inlineStr"/>
-      <c r="O98" s="4" t="inlineStr"/>
+      <c r="M98" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N98" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI05</t>
+        </is>
+      </c>
+      <c r="O98" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确运动，具名结局仅肌肉卫星细胞增殖，未列免疫细胞或组学；按 TI05 排除。</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -6420,9 +7300,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M99" s="4" t="inlineStr"/>
+      <c r="M99" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N99" s="4" t="inlineStr"/>
-      <c r="O99" s="4" t="inlineStr"/>
+      <c r="O99" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名含细胞因子表达及疾病分类分析，未明确非运动研究暴露；按 TI04 豁免推进。</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -6481,9 +7369,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M100" s="4" t="inlineStr"/>
+      <c r="M100" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N100" s="4" t="inlineStr"/>
-      <c r="O100" s="4" t="inlineStr"/>
+      <c r="O100" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅列受体蛋白及过敏反应，未明确实际暴露或来源类型；默认推进。</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -6542,9 +7438,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M101" s="4" t="inlineStr"/>
+      <c r="M101" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N101" s="4" t="inlineStr"/>
-      <c r="O101" s="4" t="inlineStr"/>
+      <c r="O101" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名含神经免疫特征及疾病表型，未明确研究暴露；临床人群与缺少运动词不足以用 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -6603,9 +7507,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M102" s="4" t="inlineStr"/>
+      <c r="M102" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N102" s="4" t="inlineStr"/>
-      <c r="O102" s="4" t="inlineStr"/>
+      <c r="O102" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅为免疫疾病的临床表现，未明确暴露；病例性质不单独构成 TI01，推进。</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -6664,9 +7576,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M103" s="4" t="inlineStr"/>
+      <c r="M103" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N103" s="4" t="inlineStr"/>
-      <c r="O103" s="4" t="inlineStr"/>
+      <c r="O103" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅描述患者危象及结局，未明示非运动研究暴露；young 及临床人群不能单独排除。</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -6725,9 +7645,17 @@
           <t>TI05</t>
         </is>
       </c>
-      <c r="M104" s="4" t="inlineStr"/>
+      <c r="M104" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N104" s="4" t="inlineStr"/>
-      <c r="O104" s="4" t="inlineStr"/>
+      <c r="O104" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确抗阻运动后 DOMS，未限定为仅酸痛评分；按运动后肌肉损伤/酸痛边界推进。</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -6786,9 +7714,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M105" s="4" t="inlineStr"/>
-      <c r="N105" s="4" t="inlineStr"/>
-      <c r="O105" s="4" t="inlineStr"/>
+      <c r="M105" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N105" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O105" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅研究堆肥提取物中大肠杆菌的生长，aerobic 指培养环境而非运动；取 TI02。</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -6847,9 +7787,21 @@
           <t>TI01</t>
         </is>
       </c>
-      <c r="M106" s="4" t="inlineStr"/>
-      <c r="N106" s="4" t="inlineStr"/>
-      <c r="O106" s="4" t="inlineStr"/>
+      <c r="M106" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N106" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI05</t>
+        </is>
+      </c>
+      <c r="O106" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名未声明综述，期刊名称不能替代文献类型；具名结局仅运动诱发支气管收缩，取 TI05。</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -6908,9 +7860,17 @@
           <t>TI03</t>
         </is>
       </c>
-      <c r="M107" s="4" t="inlineStr"/>
+      <c r="M107" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N107" s="4" t="inlineStr"/>
-      <c r="O107" s="4" t="inlineStr"/>
+      <c r="O107" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">juvenile 属疾病名称，未明示队列年龄；运动后肌肉 MR 改变可能涉及炎症，TI03/TI05 不明确。</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -6969,9 +7929,17 @@
           <t>TI05</t>
         </is>
       </c>
-      <c r="M108" s="4" t="inlineStr"/>
+      <c r="M108" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N108" s="4" t="inlineStr"/>
-      <c r="O108" s="4" t="inlineStr"/>
+      <c r="O108" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名含 DOMS，提示运动后酸痛且未限定为仅评分；TI04/TI05 不明确，保留到摘要。</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -7030,9 +7998,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M109" s="4" t="inlineStr"/>
-      <c r="N109" s="4" t="inlineStr"/>
-      <c r="O109" s="4" t="inlineStr"/>
+      <c r="M109" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N109" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O109" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确仅体外巨噬细胞吞噬实验，未列人参与者样本；TI02 优先于激素暴露的 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -7091,9 +8071,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M110" s="4" t="inlineStr"/>
+      <c r="M110" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N110" s="4" t="inlineStr"/>
-      <c r="O110" s="4" t="inlineStr"/>
+      <c r="O110" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名未限定 sudden cardiac death 的 risk factors，可能包括免疫标志物；不能确认 TI05。</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -7152,9 +8140,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M111" s="4" t="inlineStr"/>
-      <c r="N111" s="4" t="inlineStr"/>
-      <c r="O111" s="4" t="inlineStr"/>
+      <c r="M111" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N111" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI04</t>
+        </is>
+      </c>
+      <c r="O111" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">病例报告属 TI01 豁免；题名明确苯妥英药物超敏反应且无运动情境，按 TI04 排除。</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -7213,9 +8213,21 @@
           <t>TI02</t>
         </is>
       </c>
-      <c r="M112" s="4" t="inlineStr"/>
-      <c r="N112" s="4" t="inlineStr"/>
-      <c r="O112" s="4" t="inlineStr"/>
+      <c r="M112" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N112" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O112" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确 experiments with 肌腱成纤维细胞及肿瘤细胞，属仅细胞实验；取 TI02。</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -7274,9 +8286,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M113" s="4" t="inlineStr"/>
+      <c r="M113" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N113" s="4" t="inlineStr"/>
-      <c r="O113" s="4" t="inlineStr"/>
+      <c r="O113" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名含 T 细胞及人妊娠血清因子，人体样本不等于仅培养细胞；未明示非运动暴露，推进。</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -7335,9 +8355,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M114" s="4" t="inlineStr"/>
-      <c r="N114" s="4" t="inlineStr"/>
-      <c r="O114" s="4" t="inlineStr"/>
+      <c r="M114" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N114" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI04</t>
+        </is>
+      </c>
+      <c r="O114" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">human peripheral blood cultures 可为人体样本测定，TI02 不明确；辐射/咖啡因暴露明确且无运动，取 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -7396,9 +8428,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M115" s="4" t="inlineStr"/>
-      <c r="N115" s="4" t="inlineStr"/>
-      <c r="O115" s="4" t="inlineStr"/>
+      <c r="M115" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N115" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI04</t>
+        </is>
+      </c>
+      <c r="O115" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">clinicopathological exercises 指临床病例教学而非体力活动，病例记录不单独作 TI01；取 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -7457,9 +8501,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M116" s="4" t="inlineStr"/>
-      <c r="N116" s="4" t="inlineStr"/>
-      <c r="O116" s="4" t="inlineStr"/>
+      <c r="M116" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N116" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI04</t>
+        </is>
+      </c>
+      <c r="O116" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">病例报告属 TI01 豁免；题名明确色甘酸钠治疗中的反应且无运动情境，按 TI04 排除。</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -7518,9 +8574,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M117" s="4" t="inlineStr"/>
+      <c r="M117" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N117" s="4" t="inlineStr"/>
-      <c r="O117" s="4" t="inlineStr"/>
+      <c r="O117" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名未说明呼吸诊断的测试方式、实际暴露或具体测量；临床人群与缺少运动词不足以排除。</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -7579,9 +8643,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M118" s="4" t="inlineStr"/>
+      <c r="M118" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N118" s="4" t="inlineStr"/>
-      <c r="O118" s="4" t="inlineStr"/>
+      <c r="O118" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅描述炎症微环境及生物过程，未明示物种、培养细胞或实际研究暴露；默认推进。</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -7640,9 +8712,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M119" s="4" t="inlineStr"/>
+      <c r="M119" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N119" s="4" t="inlineStr"/>
-      <c r="O119" s="4" t="inlineStr"/>
+      <c r="O119" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名含 TRAF6/miR-124 及分子机制，未明示培养细胞或实际非运动干预；默认推进。</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -7701,9 +8781,21 @@
           <t>TI02</t>
         </is>
       </c>
-      <c r="M120" s="4" t="inlineStr"/>
-      <c r="N120" s="4" t="inlineStr"/>
-      <c r="O120" s="4" t="inlineStr"/>
+      <c r="M120" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N120" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O120" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确 cultured human mononuclear cells，未列人体参与者样本；TI02 优先于药物毒性的 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -7762,9 +8854,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M121" s="4" t="inlineStr"/>
+      <c r="M121" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N121" s="4" t="inlineStr"/>
-      <c r="O121" s="4" t="inlineStr"/>
+      <c r="O121" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅列基因/蛋白表达与转移关联，未明确研究暴露；临床疾病不单独作 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -7823,9 +8923,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M122" s="4" t="inlineStr"/>
+      <c r="M122" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N122" s="4" t="inlineStr"/>
-      <c r="O122" s="4" t="inlineStr"/>
+      <c r="O122" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名未列风险分层的具体指标、实际暴露或明确综述类型；无题名阶段封闭理由，推进。</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -7884,9 +8992,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M123" s="4" t="inlineStr"/>
+      <c r="M123" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N123" s="4" t="inlineStr"/>
-      <c r="O123" s="4" t="inlineStr"/>
+      <c r="O123" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅描述细胞外基质与 T 细胞功能，未明示培养或实验暴露；按 TI04 的细胞豁免推进。</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -7945,9 +9061,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M124" s="4" t="inlineStr"/>
+      <c r="M124" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N124" s="4" t="inlineStr"/>
-      <c r="O124" s="4" t="inlineStr"/>
+      <c r="O124" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅描述 T 细胞增殖及信号通路，未明确实际暴露或培养细胞；默认推进。</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -8006,9 +9130,17 @@
           <t>TI05</t>
         </is>
       </c>
-      <c r="M125" s="4" t="inlineStr"/>
+      <c r="M125" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N125" s="4" t="inlineStr"/>
-      <c r="O125" s="4" t="inlineStr"/>
+      <c r="O125" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅命名运动相关肺出血，未列具体功能/症状测量或物种；按未明确结局/人群原则推进。</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -8067,9 +9199,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M126" s="4" t="inlineStr"/>
+      <c r="M126" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N126" s="4" t="inlineStr"/>
-      <c r="O126" s="4" t="inlineStr"/>
+      <c r="O126" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅列患者的免疫疾病表现，未明示研究暴露；病例性质不单独构成 TI01。</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -8128,9 +9268,21 @@
           <t>TI02</t>
         </is>
       </c>
-      <c r="M127" s="4" t="inlineStr"/>
-      <c r="N127" s="4" t="inlineStr"/>
-      <c r="O127" s="4" t="inlineStr"/>
+      <c r="M127" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N127" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O127" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确 WEHI 231、RAJI 细胞系及脾 B 细胞实验，未列人体参与者；TI02 优先于 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -8189,9 +9341,21 @@
           <t>TI02</t>
         </is>
       </c>
-      <c r="M128" s="4" t="inlineStr"/>
-      <c r="N128" s="4" t="inlineStr"/>
-      <c r="O128" s="4" t="inlineStr"/>
+      <c r="M128" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N128" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI04</t>
+        </is>
+      </c>
+      <c r="O128" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名未明确细胞系或培养来源，TI02 不确定；X 射线辐射暴露明确且无运动情境，取 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -8250,9 +9414,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M129" s="4" t="inlineStr"/>
+      <c r="M129" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N129" s="4" t="inlineStr"/>
-      <c r="O129" s="4" t="inlineStr"/>
+      <c r="O129" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅列细胞因子、NO 合成及肝再生，未明示实际暴露或物种；默认推进。</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -8311,9 +9483,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M130" s="4" t="inlineStr"/>
+      <c r="M130" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N130" s="4" t="inlineStr"/>
-      <c r="O130" s="4" t="inlineStr"/>
+      <c r="O130" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅描述 TNF/IL-1 的分子调节，未明示外源给药或实际实验暴露；不能推定 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -8372,9 +9552,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M131" s="4" t="inlineStr"/>
+      <c r="M131" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N131" s="4" t="inlineStr"/>
-      <c r="O131" s="4" t="inlineStr"/>
+      <c r="O131" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">proliferative stimulus 来源未明，题名含胸腺细胞及蛋白；不能确认仅培养或非运动暴露。</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -8433,9 +9621,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M132" s="4" t="inlineStr"/>
+      <c r="M132" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N132" s="4" t="inlineStr"/>
-      <c r="O132" s="4" t="inlineStr"/>
+      <c r="O132" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅列正常人 T 细胞中的蛋白调节及细胞周期，未明确培养或实际暴露；默认推进。</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -8494,9 +9690,21 @@
           <t>TI02</t>
         </is>
       </c>
-      <c r="M133" s="4" t="inlineStr"/>
-      <c r="N133" s="4" t="inlineStr"/>
-      <c r="O133" s="4" t="inlineStr"/>
+      <c r="M133" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N133" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O133" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确 memory T-cell activation in vitro，未列人体参与者样本；按仅体外细胞实验取 TI02。</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -8555,9 +9763,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M134" s="4" t="inlineStr"/>
+      <c r="M134" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N134" s="4" t="inlineStr"/>
-      <c r="O134" s="4" t="inlineStr"/>
+      <c r="O134" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名未明确实际暴露、具体测量或综述类型；疾病群体与病理框架描述不单独构成排除理由。</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -8616,9 +9832,17 @@
           <t>TI05</t>
         </is>
       </c>
-      <c r="M135" s="4" t="inlineStr"/>
+      <c r="M135" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N135" s="4" t="inlineStr"/>
-      <c r="O135" s="4" t="inlineStr"/>
+      <c r="O135" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确 exercise-triggered irisin，未限定为仅焦虑评分；按可能相关蛋白的 TI05 豁免推进。</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -8677,9 +9901,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M136" s="4" t="inlineStr"/>
+      <c r="M136" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N136" s="4" t="inlineStr"/>
-      <c r="O136" s="4" t="inlineStr"/>
+      <c r="O136" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅比较食物过敏/过敏反应与族群，未明示实际研究暴露；按 TI04 豁免推进。</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -8738,9 +9970,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M137" s="4" t="inlineStr"/>
-      <c r="N137" s="4" t="inlineStr"/>
-      <c r="O137" s="4" t="inlineStr"/>
+      <c r="M137" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N137" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O137" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确褐藻生命周期中的线粒体形态，研究对象仅非人类生物；取 TI02。</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -8799,9 +10043,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M138" s="4" t="inlineStr"/>
-      <c r="N138" s="4" t="inlineStr"/>
-      <c r="O138" s="4" t="inlineStr"/>
+      <c r="M138" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N138" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O138" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确沙门菌在腐殖酸条件下的回收，recovery 非人体恢复；TI02 优先于 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -8852,9 +10108,21 @@
           <t>TI01</t>
         </is>
       </c>
-      <c r="M139" s="4" t="inlineStr"/>
-      <c r="N139" s="4" t="inlineStr"/>
-      <c r="O139" s="4" t="inlineStr"/>
+      <c r="M139" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N139" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI01</t>
+        </is>
+      </c>
+      <c r="O139" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">COUNTERPOINT 及 REBUTTAL 明确为观点辩论/评论文体；按 TI01 排除。</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -8913,9 +10181,21 @@
           <t>TI02</t>
         </is>
       </c>
-      <c r="M140" s="4" t="inlineStr"/>
-      <c r="N140" s="4" t="inlineStr"/>
-      <c r="O140" s="4" t="inlineStr"/>
+      <c r="M140" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N140" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O140" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确人骨髓瘤细胞的凋亡实验，未列人体参与者；TI02 优先于蛋白刺激的 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -8974,9 +10254,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M141" s="4" t="inlineStr"/>
-      <c r="N141" s="4" t="inlineStr"/>
-      <c r="O141" s="4" t="inlineStr"/>
+      <c r="M141" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N141" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O141" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确 Caulobacter 细菌的细胞周期及 FtsZ 调节，研究对象仅非人类；取 TI02。</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -9035,9 +10327,21 @@
           <t>TI02</t>
         </is>
       </c>
-      <c r="M142" s="4" t="inlineStr"/>
-      <c r="N142" s="4" t="inlineStr"/>
-      <c r="O142" s="4" t="inlineStr"/>
+      <c r="M142" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N142" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O142" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确 IL-1 对人黑色素瘤细胞的生长抑制实验，未列人体参与者；TI02 优先于 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -9096,9 +10400,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M143" s="4" t="inlineStr"/>
+      <c r="M143" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N143" s="4" t="inlineStr"/>
-      <c r="O143" s="4" t="inlineStr"/>
+      <c r="O143" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅描述 IL-1β 与 LIF 转录调节，未明示给药、培养细胞或实际实验暴露；默认推进。</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -9157,9 +10469,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M144" s="4" t="inlineStr"/>
+      <c r="M144" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N144" s="4" t="inlineStr"/>
-      <c r="O144" s="4" t="inlineStr"/>
+      <c r="O144" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名测量胚胎培养液中的免疫因子，可来自人临床样本；未明确仅非人类/细胞或非运动暴露。</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -9210,9 +10530,17 @@
           <t>TI02</t>
         </is>
       </c>
-      <c r="M145" s="4" t="inlineStr"/>
+      <c r="M145" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N145" s="4" t="inlineStr"/>
-      <c r="O145" s="4" t="inlineStr"/>
+      <c r="O145" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">人体白细胞的体外测定可能来自人参与者样本，诱发因素未限定；TI02/TI04 不明确。</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -9271,9 +10599,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M146" s="4" t="inlineStr"/>
+      <c r="M146" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N146" s="4" t="inlineStr"/>
-      <c r="O146" s="4" t="inlineStr"/>
+      <c r="O146" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅描述淋巴细胞调节物及 DNA 合成机制，未明示培养或实际外源刺激；默认推进。</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -9332,9 +10668,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M147" s="4" t="inlineStr"/>
-      <c r="N147" s="4" t="inlineStr"/>
-      <c r="O147" s="4" t="inlineStr"/>
+      <c r="M147" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N147" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O147" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名研究对象为伯氏疏螺旋体分离株，human complement 指试剂来源而非人队列；取 TI02。</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -9393,9 +10741,21 @@
           <t>TI02</t>
         </is>
       </c>
-      <c r="M148" s="4" t="inlineStr"/>
-      <c r="N148" s="4" t="inlineStr"/>
-      <c r="O148" s="4" t="inlineStr"/>
+      <c r="M148" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N148" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O148" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确瘤胃上皮细胞，属于非人类组织/细胞实验；TI02 优先于基因过表达的 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -9454,9 +10814,21 @@
           <t>TI05</t>
         </is>
       </c>
-      <c r="M149" s="4" t="inlineStr"/>
-      <c r="N149" s="4" t="inlineStr"/>
-      <c r="O149" s="4" t="inlineStr"/>
+      <c r="M149" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N149" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI05</t>
+        </is>
+      </c>
+      <c r="O149" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DOMS 提供运动后情境，TI04 不成立；具名结局仅疼痛、压痛及肌肉僵硬，按症状边界取 TI05。</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -9515,9 +10887,17 @@
           <t>TI02</t>
         </is>
       </c>
-      <c r="M150" s="4" t="inlineStr"/>
+      <c r="M150" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N150" s="4" t="inlineStr"/>
-      <c r="O150" s="4" t="inlineStr"/>
+      <c r="O150" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确 AKI 患者尿液样本及细胞模型，非仅培养细胞；未明示非运动研究暴露，推进。</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -9576,9 +10956,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M151" s="4" t="inlineStr"/>
-      <c r="N151" s="4" t="inlineStr"/>
-      <c r="O151" s="4" t="inlineStr"/>
+      <c r="M151" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N151" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O151" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确熟肉食品的细菌灭活，研究对象为非人体食品/微生物；TI02 优先于 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -9637,9 +11029,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M152" s="4" t="inlineStr"/>
+      <c r="M152" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N152" s="4" t="inlineStr"/>
-      <c r="O152" s="4" t="inlineStr"/>
+      <c r="O152" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅描述 irisin 与炎症信号通路，未明示外源给药或实际实验暴露；不能推定 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -9698,9 +11098,21 @@
           <t>TI02</t>
         </is>
       </c>
-      <c r="M153" s="4" t="inlineStr"/>
-      <c r="N153" s="4" t="inlineStr"/>
-      <c r="O153" s="4" t="inlineStr"/>
+      <c r="M153" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N153" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O153" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确人胰腺癌细胞的药物细胞毒性实验，未列人体参与者；TI02 优先于 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -9759,9 +11171,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M154" s="4" t="inlineStr"/>
+      <c r="M154" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N154" s="4" t="inlineStr"/>
-      <c r="O154" s="4" t="inlineStr"/>
+      <c r="O154" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅列 ASB9、卵巢细胞功能及信号通路，未明确培养、物种或实际研究暴露；默认推进。</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -9820,9 +11240,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M155" s="4" t="inlineStr"/>
-      <c r="N155" s="4" t="inlineStr"/>
-      <c r="O155" s="4" t="inlineStr"/>
+      <c r="M155" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N155" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O155" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确利什曼原虫的前鞭毛体/无鞭毛体，研究对象仅非人类；TI02 优先于化合物的 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -9881,9 +11313,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M156" s="4" t="inlineStr"/>
+      <c r="M156" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N156" s="4" t="inlineStr"/>
-      <c r="O156" s="4" t="inlineStr"/>
+      <c r="O156" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅列患者的节律基因表达，未明示研究暴露；临床人群及缺少运动词不足以用 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -9942,9 +11382,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M157" s="4" t="inlineStr"/>
+      <c r="M157" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N157" s="4" t="inlineStr"/>
-      <c r="O157" s="4" t="inlineStr"/>
+      <c r="O157" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名未说明问卷项目、队列年龄或具体暴露，不能凭缩写猜测排除条件；默认推进。</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -10003,9 +11451,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M158" s="4" t="inlineStr"/>
+      <c r="M158" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N158" s="4" t="inlineStr"/>
-      <c r="O158" s="4" t="inlineStr"/>
+      <c r="O158" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅列基因缺失及细胞分裂机制，未明示物种、培养细胞或实际实验暴露；默认推进。</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -10064,9 +11520,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M159" s="4" t="inlineStr"/>
-      <c r="N159" s="4" t="inlineStr"/>
-      <c r="O159" s="4" t="inlineStr"/>
+      <c r="M159" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N159" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O159" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确仅体外 HIV-1 复制抑制，human 属病毒名称而非人体参与者；TI02 优先于 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -10125,9 +11593,17 @@
           <t>TI05</t>
         </is>
       </c>
-      <c r="M160" s="4" t="inlineStr"/>
+      <c r="M160" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N160" s="4" t="inlineStr"/>
-      <c r="O160" s="4" t="inlineStr"/>
+      <c r="O160" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅描述 VEGF 蛋白与骨骼肌血管生成/血流，未明确研究暴露；按 TI04 豁免推进。</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -10186,9 +11662,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M161" s="4" t="inlineStr"/>
+      <c r="M161" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N161" s="4" t="inlineStr"/>
-      <c r="O161" s="4" t="inlineStr"/>
+      <c r="O161" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名含黄体转录组及内源介质反应，未明示外源给药或物种；不能确认 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -10247,9 +11731,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M162" s="4" t="inlineStr"/>
-      <c r="N162" s="4" t="inlineStr"/>
-      <c r="O162" s="4" t="inlineStr"/>
+      <c r="M162" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N162" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O162" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确 Ashbya 真菌菌丝的胞质分裂，研究对象仅非人类；取 TI02。</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -10308,9 +11804,21 @@
           <t>TI02</t>
         </is>
       </c>
-      <c r="M163" s="4" t="inlineStr"/>
-      <c r="N163" s="4" t="inlineStr"/>
-      <c r="O163" s="4" t="inlineStr"/>
+      <c r="M163" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N163" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O163" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确耐放射肿瘤细胞的药物/辐射实验，未列人体参与者；TI02 优先于 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -10369,9 +11877,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M164" s="4" t="inlineStr"/>
-      <c r="N164" s="4" t="inlineStr"/>
-      <c r="O164" s="4" t="inlineStr"/>
+      <c r="M164" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N164" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI04</t>
+        </is>
+      </c>
+      <c r="O164" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">人体淋巴细胞可来自人样本，TI02 不明确；题名明确阿维 A/抗肿瘤药暴露且无运动，取 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -10430,9 +11950,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M165" s="4" t="inlineStr"/>
-      <c r="N165" s="4" t="inlineStr"/>
-      <c r="O165" s="4" t="inlineStr"/>
+      <c r="M165" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N165" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O165" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确链霉菌的酶活性，complement 指酶系组成而非人体免疫测量；取 TI02。</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
@@ -10491,9 +12023,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M166" s="4" t="inlineStr"/>
-      <c r="N166" s="4" t="inlineStr"/>
-      <c r="O166" s="4" t="inlineStr"/>
+      <c r="M166" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N166" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O166" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确克氏锥虫生活史转换的基因表达，研究对象仅寄生虫；取 TI02。</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
@@ -10552,9 +12096,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M167" s="4" t="inlineStr"/>
+      <c r="M167" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N167" s="4" t="inlineStr"/>
-      <c r="O167" s="4" t="inlineStr"/>
+      <c r="O167" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅描述蛋白磷酸化与有丝分裂，未明示物种、培养细胞或实际研究暴露；默认推进。</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
@@ -10613,9 +12165,21 @@
           <t>TI02</t>
         </is>
       </c>
-      <c r="M168" s="4" t="inlineStr"/>
-      <c r="N168" s="4" t="inlineStr"/>
-      <c r="O168" s="4" t="inlineStr"/>
+      <c r="M168" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N168" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O168" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅列大鼠及人的胶质瘤细胞实验，human cells 不等于人体参与者；TI02 优先于 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -10674,9 +12238,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M169" s="4" t="inlineStr"/>
-      <c r="N169" s="4" t="inlineStr"/>
-      <c r="O169" s="4" t="inlineStr"/>
+      <c r="M169" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N169" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O169" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确细菌产物用于肉类去污染及保藏，研究对象为食品/微生物而非人；取 TI02。</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
@@ -10735,9 +12311,21 @@
           <t>TI02</t>
         </is>
       </c>
-      <c r="M170" s="4" t="inlineStr"/>
-      <c r="N170" s="4" t="inlineStr"/>
-      <c r="O170" s="4" t="inlineStr"/>
+      <c r="M170" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N170" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O170" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确人卵巢癌细胞的药物细胞毒性实验，未列人体参与者；TI02 优先于 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -10796,9 +12384,21 @@
           <t>TI02</t>
         </is>
       </c>
-      <c r="M171" s="4" t="inlineStr"/>
-      <c r="N171" s="4" t="inlineStr"/>
-      <c r="O171" s="4" t="inlineStr"/>
+      <c r="M171" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N171" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O171" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确激酶表达细胞的药物杀伤比较，未列人体参与者；TI02 优先于 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
@@ -10857,9 +12457,17 @@
           <t>TI02</t>
         </is>
       </c>
-      <c r="M172" s="4" t="inlineStr"/>
+      <c r="M172" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N172" s="4" t="inlineStr"/>
-      <c r="O172" s="4" t="inlineStr"/>
+      <c r="O172" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅描述 Oncostatin M 与内皮细胞的分子功能，未明示培养或实际给药暴露；默认推进。</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
@@ -10918,9 +12526,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M173" s="4" t="inlineStr"/>
-      <c r="N173" s="4" t="inlineStr"/>
-      <c r="O173" s="4" t="inlineStr"/>
+      <c r="M173" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N173" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O173" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确疱疹病毒基因组结构，human 属病毒名称而非人体队列；取 TI02。</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
@@ -10979,9 +12599,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M174" s="4" t="inlineStr"/>
+      <c r="M174" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N174" s="4" t="inlineStr"/>
-      <c r="O174" s="4" t="inlineStr"/>
+      <c r="O174" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅描述干扰素与细胞周期基因调节，未明示给药、培养细胞或实际实验暴露；默认推进。</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
@@ -11040,9 +12668,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M175" s="4" t="inlineStr"/>
+      <c r="M175" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N175" s="4" t="inlineStr"/>
-      <c r="O175" s="4" t="inlineStr"/>
+      <c r="O175" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ovine 指蛋白来源，不能证明研究对象仅动物；题名未明确培养或实际暴露，TI02/TI04 不明确。</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
@@ -11101,9 +12737,17 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M176" s="4" t="inlineStr"/>
+      <c r="M176" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADVANCE_TO_ABSTRACT</t>
+        </is>
+      </c>
       <c r="N176" s="4" t="inlineStr"/>
-      <c r="O176" s="4" t="inlineStr"/>
+      <c r="O176" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名仅描述免疫介质与正常人单核细胞的基因反应，未明示培养或外源给药；默认推进。</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
@@ -11162,9 +12806,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M177" s="4" t="inlineStr"/>
-      <c r="N177" s="4" t="inlineStr"/>
-      <c r="O177" s="4" t="inlineStr"/>
+      <c r="M177" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N177" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O177" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确李斯特菌的附着生长及清洁剂/热耐受，研究对象仅细菌；TI02 优先于 TI04。</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
@@ -11223,9 +12879,21 @@
           <t>TI04</t>
         </is>
       </c>
-      <c r="M178" s="4" t="inlineStr"/>
-      <c r="N178" s="4" t="inlineStr"/>
-      <c r="O178" s="4" t="inlineStr"/>
+      <c r="M178" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUDE_TITLE</t>
+        </is>
+      </c>
+      <c r="N178" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TI02</t>
+        </is>
+      </c>
+      <c r="O178" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题名明确即食生菜上的李斯特菌，研究对象为食品/微生物而非人；取 TI02。</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="2">

</xml_diff>